<commit_message>
new Agile project added
</commit_message>
<xml_diff>
--- a/Guru99/src/test/resources/agileTest.xlsx
+++ b/Guru99/src/test/resources/agileTest.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Axis\git\repository\Guru99App\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67BBD478-F084-4203-9D27-C08A9D82EA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6A599B6B-D108-4C38-9987-77AF884E701A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4824" yWindow="5952" windowWidth="17928" windowHeight="6288" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>UserID</t>
   </si>
@@ -514,12 +510,8 @@
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
-        <v>1303</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>5</v>
-      </c>
+      <c r="A4" s="5"/>
+      <c r="B4" s="7"/>
       <c r="C4" s="2" t="s">
         <v>4</v>
       </c>

</xml_diff>